<commit_message>
Updating with duration refactoring metrics
</commit_message>
<xml_diff>
--- a/RQ1 - Refactoring Metrics.xlsx
+++ b/RQ1 - Refactoring Metrics.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Dell\Desktop\Software Testing, Quality Assurance &amp; Maintainence\Project\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{3FEFBFD1-4DF3-4158-BEFE-BC03C41CC034}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2E5CF0FA-1B7A-45E3-840F-0513CB0D4965}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="4" activeTab="7" xr2:uid="{FFC2C0CC-8ED1-41E2-BF92-62697309D203}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="5" activeTab="8" xr2:uid="{FFC2C0CC-8ED1-41E2-BF92-62697309D203}"/>
   </bookViews>
   <sheets>
     <sheet name="RQ1 - Reviewers queries" sheetId="1" r:id="rId1"/>
@@ -21,6 +21,7 @@
     <sheet name="RQ1 - Files Queries" sheetId="6" r:id="rId6"/>
     <sheet name="RQ1 -  Revisisons Queries" sheetId="7" r:id="rId7"/>
     <sheet name="RQ1 - Code Churn Queries" sheetId="8" r:id="rId8"/>
+    <sheet name="RQ1 - Duration Queries" sheetId="9" r:id="rId9"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -32,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="6">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="54" uniqueCount="6">
   <si>
     <t>Mean</t>
   </si>
@@ -938,4 +939,70 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AFC04937-8CF6-4375-87EE-A27156A5B7E2}">
+  <dimension ref="A1:C11"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="13.88671875" customWidth="1"/>
+    <col min="3" max="3" width="16.5546875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A2" s="2">
+        <v>3.0555555555555601E-3</v>
+      </c>
+      <c r="B2" s="2">
+        <v>995.05872231686601</v>
+      </c>
+      <c r="C2" s="2">
+        <v>66766.176388888896</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A4" s="1" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A5" s="2">
+        <v>3.0555555555555601E-3</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A7" s="1" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A8" s="2">
+        <v>14.3225</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A10" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A11" s="2">
+        <v>314.39166666666699</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>